<commit_message>
regen pre-survey data for clean 6-factor PCA; each dimension maps to distinct factor
Agent-Logs-Url: https://github.com/via-zy/SEM-fsQCA/sessions/024b65cd-8c8e-4358-ad3e-827f7223dce0

Co-authored-by: via-zy <216556376+via-zy@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/预调研问卷可行性数据.xlsx
+++ b/预调研问卷可行性数据.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="预调研数据" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="信效度分析结果" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="预调研数据" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="信效度分析结果" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -579,58 +579,58 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="S2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="T2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="X2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -668,58 +668,58 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="U3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="W3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="X3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Y3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -757,40 +757,40 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T4" t="n">
         <v>2</v>
@@ -802,13 +802,13 @@
         <v>2</v>
       </c>
       <c r="W4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -846,58 +846,58 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W5" t="n">
         <v>4</v>
       </c>
       <c r="X5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Y5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -935,58 +935,58 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I6" t="n">
         <v>3</v>
       </c>
       <c r="J6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O6" t="n">
         <v>4</v>
       </c>
       <c r="P6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q6" t="n">
         <v>3</v>
       </c>
       <c r="R6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="X6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Y6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -1024,16 +1024,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L7" t="n">
         <v>4</v>
@@ -1042,22 +1042,22 @@
         <v>5</v>
       </c>
       <c r="N7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T7" t="n">
         <v>3</v>
@@ -1066,16 +1066,16 @@
         <v>4</v>
       </c>
       <c r="V7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W7" t="n">
         <v>3</v>
       </c>
       <c r="X7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Y7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -1113,43 +1113,43 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P8" t="n">
         <v>3</v>
       </c>
       <c r="Q8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U8" t="n">
         <v>3</v>
@@ -1161,10 +1161,10 @@
         <v>3</v>
       </c>
       <c r="X8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Y8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -1202,16 +1202,16 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L9" t="n">
         <v>4</v>
@@ -1220,40 +1220,40 @@
         <v>4</v>
       </c>
       <c r="N9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="X9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Y9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1291,7 +1291,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I10" t="n">
         <v>2</v>
@@ -1300,46 +1300,46 @@
         <v>2</v>
       </c>
       <c r="K10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V10" t="n">
         <v>3</v>
       </c>
       <c r="W10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y10" t="n">
         <v>2</v>
@@ -1383,40 +1383,40 @@
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O11" t="n">
         <v>1</v>
       </c>
       <c r="P11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S11" t="n">
         <v>3</v>
       </c>
       <c r="T11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U11" t="n">
         <v>3</v>
@@ -1425,13 +1425,13 @@
         <v>3</v>
       </c>
       <c r="W11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="X11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Y11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -1469,58 +1469,58 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J12" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K12" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M12" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W12" t="n">
         <v>5</v>
       </c>
       <c r="X12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Y12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -1561,55 +1561,55 @@
         <v>3</v>
       </c>
       <c r="I13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R13" t="n">
         <v>3</v>
       </c>
       <c r="S13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V13" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="W13" t="n">
         <v>3</v>
       </c>
       <c r="X13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Y13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1647,55 +1647,55 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I14" t="n">
         <v>3</v>
       </c>
       <c r="J14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M14" t="n">
         <v>3</v>
       </c>
       <c r="N14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P14" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q14" t="n">
         <v>2</v>
       </c>
       <c r="R14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S14" t="n">
         <v>3</v>
       </c>
       <c r="T14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V14" t="n">
         <v>3</v>
       </c>
       <c r="W14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Y14" t="n">
         <v>3</v>
@@ -1736,58 +1736,58 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M15" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N15" t="n">
         <v>5</v>
       </c>
       <c r="O15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="n">
         <v>3</v>
       </c>
       <c r="V15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="X15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Y15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -1825,58 +1825,58 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q16" t="n">
         <v>3</v>
       </c>
       <c r="R16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T16" t="n">
         <v>2</v>
       </c>
       <c r="U16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W16" t="n">
         <v>3</v>
       </c>
       <c r="X16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Y16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -1914,40 +1914,40 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K17" t="n">
         <v>2</v>
       </c>
       <c r="L17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q17" t="n">
         <v>2</v>
       </c>
       <c r="R17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T17" t="n">
         <v>4</v>
@@ -1962,10 +1962,10 @@
         <v>3</v>
       </c>
       <c r="X17" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Y17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -2003,46 +2003,46 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I18" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K18" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M18" t="n">
         <v>4</v>
       </c>
       <c r="N18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O18" t="n">
         <v>3</v>
       </c>
       <c r="P18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V18" t="n">
         <v>3</v>
@@ -2051,10 +2051,10 @@
         <v>3</v>
       </c>
       <c r="X18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Y18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
@@ -2095,16 +2095,16 @@
         <v>3</v>
       </c>
       <c r="I19" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M19" t="n">
         <v>3</v>
@@ -2119,31 +2119,31 @@
         <v>2</v>
       </c>
       <c r="Q19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R19" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T19" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U19" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V19" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="W19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X19" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Y19" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -2181,58 +2181,58 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J20" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K20" t="n">
         <v>3</v>
       </c>
       <c r="L20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O20" t="n">
         <v>4</v>
       </c>
       <c r="P20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="X20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Y20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -2270,58 +2270,58 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N21" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P21" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R21" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T21" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="U21" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V21" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="W21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="X21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y21" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
@@ -2359,7 +2359,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I22" t="n">
         <v>3</v>
@@ -2374,19 +2374,19 @@
         <v>3</v>
       </c>
       <c r="M22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N22" t="n">
         <v>4</v>
       </c>
       <c r="O22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P22" t="n">
         <v>4</v>
       </c>
       <c r="Q22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R22" t="n">
         <v>3</v>
@@ -2398,16 +2398,16 @@
         <v>4</v>
       </c>
       <c r="U22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W22" t="n">
         <v>4</v>
       </c>
       <c r="X22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Y22" t="n">
         <v>4</v>
@@ -2448,22 +2448,22 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N23" t="n">
         <v>2</v>
@@ -2472,25 +2472,25 @@
         <v>3</v>
       </c>
       <c r="P23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q23" t="n">
         <v>3</v>
       </c>
       <c r="R23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="W23" t="n">
         <v>2</v>
@@ -2499,7 +2499,7 @@
         <v>3</v>
       </c>
       <c r="Y23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -2537,58 +2537,58 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q24" t="n">
         <v>3</v>
       </c>
       <c r="R24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="X24" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Y24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -2626,16 +2626,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L25" t="n">
         <v>3</v>
@@ -2644,31 +2644,31 @@
         <v>3</v>
       </c>
       <c r="N25" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S25" t="n">
         <v>2</v>
       </c>
       <c r="T25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U25" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V25" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W25" t="n">
         <v>3</v>
@@ -2715,34 +2715,34 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I26" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J26" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L26" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N26" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O26" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P26" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R26" t="n">
         <v>3</v>
@@ -2751,16 +2751,16 @@
         <v>4</v>
       </c>
       <c r="T26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W26" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="X26" t="n">
         <v>4</v>
@@ -2804,34 +2804,34 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I27" t="n">
         <v>2</v>
       </c>
       <c r="J27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L27" t="n">
         <v>2</v>
       </c>
       <c r="M27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N27" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O27" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P27" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R27" t="n">
         <v>2</v>
@@ -2840,22 +2840,22 @@
         <v>2</v>
       </c>
       <c r="T27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V27" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="W27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X27" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Y27" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28">
@@ -2896,55 +2896,55 @@
         <v>4</v>
       </c>
       <c r="I28" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J28" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K28" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L28" t="n">
         <v>3</v>
       </c>
       <c r="M28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P28" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R28" t="n">
         <v>2</v>
       </c>
       <c r="S28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T28" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V28" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="W28" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="X28" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Y28" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29">
@@ -2985,34 +2985,34 @@
         <v>4</v>
       </c>
       <c r="I29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J29" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K29" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L29" t="n">
         <v>3</v>
       </c>
       <c r="M29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P29" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q29" t="n">
         <v>3</v>
       </c>
       <c r="R29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S29" t="n">
         <v>4</v>
@@ -3033,7 +3033,7 @@
         <v>4</v>
       </c>
       <c r="Y29" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30">
@@ -3071,43 +3071,43 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I30" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N30" t="n">
         <v>2</v>
       </c>
       <c r="O30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P30" t="n">
         <v>3</v>
       </c>
       <c r="Q30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S30" t="n">
         <v>2</v>
       </c>
       <c r="T30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U30" t="n">
         <v>2</v>
@@ -3119,7 +3119,7 @@
         <v>2</v>
       </c>
       <c r="X30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y30" t="n">
         <v>2</v>
@@ -3160,19 +3160,19 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I31" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J31" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K31" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L31" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M31" t="n">
         <v>3</v>
@@ -3181,19 +3181,19 @@
         <v>3</v>
       </c>
       <c r="O31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P31" t="n">
         <v>3</v>
       </c>
       <c r="Q31" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T31" t="n">
         <v>3</v>
@@ -3202,16 +3202,16 @@
         <v>4</v>
       </c>
       <c r="V31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W31" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="X31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Y31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
@@ -3249,58 +3249,58 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J32" t="n">
         <v>2</v>
       </c>
       <c r="K32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L32" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M32" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O32" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q32" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="R32" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S32" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T32" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U32" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V32" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="W32" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="X32" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Y32" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33">
@@ -3338,34 +3338,34 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M33" t="n">
         <v>4</v>
       </c>
       <c r="N33" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O33" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="P33" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R33" t="n">
         <v>3</v>
@@ -3374,22 +3374,22 @@
         <v>3</v>
       </c>
       <c r="T33" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="U33" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V33" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W33" t="n">
         <v>5</v>
       </c>
       <c r="X33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Y33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34">
@@ -3427,7 +3427,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I34" t="n">
         <v>3</v>
@@ -3439,7 +3439,7 @@
         <v>2</v>
       </c>
       <c r="L34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M34" t="n">
         <v>3</v>
@@ -3451,34 +3451,34 @@
         <v>4</v>
       </c>
       <c r="P34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="W34" t="n">
         <v>4</v>
       </c>
       <c r="X34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Y34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
@@ -3516,52 +3516,52 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I35" t="n">
         <v>4</v>
       </c>
       <c r="J35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M35" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N35" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O35" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P35" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R35" t="n">
         <v>4</v>
       </c>
       <c r="S35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T35" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="U35" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V35" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="W35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="X35" t="n">
         <v>5</v>
@@ -3605,58 +3605,58 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I36" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J36" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K36" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L36" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M36" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="N36" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P36" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q36" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R36" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S36" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="T36" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U36" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V36" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X36" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Y36" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
@@ -3700,13 +3700,13 @@
         <v>5</v>
       </c>
       <c r="J37" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M37" t="n">
         <v>5</v>
@@ -3715,13 +3715,13 @@
         <v>5</v>
       </c>
       <c r="O37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P37" t="n">
         <v>5</v>
       </c>
       <c r="Q37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R37" t="n">
         <v>5</v>
@@ -3730,22 +3730,22 @@
         <v>5</v>
       </c>
       <c r="T37" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V37" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W37" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="X37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Y37" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
@@ -3783,7 +3783,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I38" t="n">
         <v>4</v>
@@ -3792,25 +3792,25 @@
         <v>4</v>
       </c>
       <c r="K38" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M38" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N38" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P38" t="n">
         <v>4</v>
       </c>
       <c r="Q38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R38" t="n">
         <v>5</v>
@@ -3822,7 +3822,7 @@
         <v>4</v>
       </c>
       <c r="U38" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V38" t="n">
         <v>4</v>
@@ -3834,7 +3834,7 @@
         <v>4</v>
       </c>
       <c r="Y38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39">
@@ -3872,10 +3872,10 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J39" t="n">
         <v>2</v>
@@ -3884,13 +3884,13 @@
         <v>2</v>
       </c>
       <c r="L39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M39" t="n">
         <v>3</v>
       </c>
       <c r="N39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O39" t="n">
         <v>3</v>
@@ -3899,31 +3899,31 @@
         <v>3</v>
       </c>
       <c r="Q39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T39" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U39" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V39" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="W39" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="X39" t="n">
         <v>4</v>
       </c>
       <c r="Y39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="40">
@@ -3961,13 +3961,13 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J40" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K40" t="n">
         <v>3</v>
@@ -3976,43 +3976,43 @@
         <v>3</v>
       </c>
       <c r="M40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q40" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S40" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U40" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V40" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W40" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="X40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Y40" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41">
@@ -4053,40 +4053,40 @@
         <v>3</v>
       </c>
       <c r="I41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J41" t="n">
         <v>2</v>
       </c>
       <c r="K41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N41" t="n">
         <v>3</v>
       </c>
       <c r="O41" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P41" t="n">
         <v>3</v>
       </c>
       <c r="Q41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S41" t="n">
         <v>3</v>
       </c>
       <c r="T41" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U41" t="n">
         <v>3</v>
@@ -4095,13 +4095,13 @@
         <v>3</v>
       </c>
       <c r="W41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y41" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42">
@@ -4142,52 +4142,52 @@
         <v>3</v>
       </c>
       <c r="I42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K42" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M42" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N42" t="n">
         <v>4</v>
       </c>
       <c r="O42" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P42" t="n">
         <v>4</v>
       </c>
       <c r="Q42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T42" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W42" t="n">
         <v>3</v>
       </c>
       <c r="X42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Y42" t="n">
         <v>4</v>
@@ -4228,58 +4228,58 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I43" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J43" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L43" t="n">
         <v>4</v>
       </c>
       <c r="M43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N43" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P43" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q43" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S43" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T43" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V43" t="n">
         <v>4</v>
       </c>
       <c r="W43" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="X43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Y43" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44">
@@ -4320,43 +4320,43 @@
         <v>4</v>
       </c>
       <c r="I44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J44" t="n">
         <v>3</v>
       </c>
       <c r="K44" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L44" t="n">
         <v>3</v>
       </c>
       <c r="M44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N44" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O44" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P44" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q44" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S44" t="n">
         <v>4</v>
       </c>
       <c r="T44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V44" t="n">
         <v>4</v>
@@ -4365,10 +4365,10 @@
         <v>4</v>
       </c>
       <c r="X44" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45">
@@ -4406,7 +4406,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I45" t="n">
         <v>1</v>
@@ -4415,13 +4415,13 @@
         <v>1</v>
       </c>
       <c r="K45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L45" t="n">
         <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N45" t="n">
         <v>2</v>
@@ -4433,31 +4433,31 @@
         <v>2</v>
       </c>
       <c r="Q45" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T45" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="U45" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V45" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="W45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y45" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46">
@@ -4495,13 +4495,13 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J46" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K46" t="n">
         <v>2</v>
@@ -4510,37 +4510,37 @@
         <v>3</v>
       </c>
       <c r="M46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N46" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O46" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P46" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R46" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S46" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U46" t="n">
         <v>3</v>
       </c>
       <c r="V46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X46" t="n">
         <v>3</v>
@@ -4590,31 +4590,31 @@
         <v>3</v>
       </c>
       <c r="J47" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K47" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L47" t="n">
         <v>3</v>
       </c>
       <c r="M47" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R47" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S47" t="n">
         <v>3</v>
@@ -4623,19 +4623,19 @@
         <v>3</v>
       </c>
       <c r="U47" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V47" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Y47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48">
@@ -4673,58 +4673,58 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I48" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J48" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M48" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N48" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O48" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P48" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q48" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R48" t="n">
         <v>4</v>
       </c>
       <c r="S48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T48" t="n">
         <v>3</v>
       </c>
       <c r="U48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="X48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Y48" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49">
@@ -4762,58 +4762,58 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I49" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J49" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L49" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M49" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N49" t="n">
         <v>4</v>
       </c>
       <c r="O49" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P49" t="n">
         <v>4</v>
       </c>
       <c r="Q49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T49" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U49" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V49" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="W49" t="n">
         <v>4</v>
       </c>
       <c r="X49" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y49" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -4851,58 +4851,58 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I50" t="n">
         <v>4</v>
       </c>
       <c r="J50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K50" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L50" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M50" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O50" t="n">
         <v>4</v>
       </c>
       <c r="P50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q50" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R50" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S50" t="n">
         <v>4</v>
       </c>
       <c r="T50" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U50" t="n">
         <v>1</v>
       </c>
       <c r="V50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X50" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Y50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="51">
@@ -4940,13 +4940,13 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I51" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J51" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K51" t="n">
         <v>1</v>
@@ -4955,43 +4955,43 @@
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N51" t="n">
         <v>2</v>
       </c>
       <c r="O51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P51" t="n">
         <v>1</v>
       </c>
       <c r="Q51" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R51" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S51" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T51" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U51" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V51" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W51" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="X51" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Y51" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -5032,7 +5032,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8895</v>
+        <v>0.7352</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -5047,7 +5047,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>916.023</v>
+        <v>563.024</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -5072,6 +5072,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -5096,7 +5097,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.9255</v>
+        <v>0.891</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -5111,7 +5112,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.8632</v>
+        <v>0.858</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -5126,7 +5127,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.8897</v>
+        <v>0.904</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -5141,7 +5142,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.8937</v>
+        <v>0.838</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -5156,7 +5157,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.8593</v>
+        <v>0.902</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -5171,7 +5172,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.8552999999999999</v>
+        <v>0.889</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>

</xml_diff>